<commit_message>
KCDB_query_country_all_V1.xlsx github link added
</commit_message>
<xml_diff>
--- a/Excel/KCDB_query_country_all_V1.xlsx
+++ b/Excel/KCDB_query_country_all_V1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\CMO\Reporting\2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF7BFB84-7654-44FC-8878-C4F7316D998D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C05FF78-3B86-4C31-BEEF-215D974BF4F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{8C3526C0-0719-4BDC-A80A-CB064B81EFFC}"/>
   </bookViews>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1111" uniqueCount="444">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1113" uniqueCount="446">
   <si>
     <t>https://www.bipm.org/api/kcdb/cmc/searchData/physics</t>
   </si>
@@ -1392,6 +1392,12 @@
   </si>
   <si>
     <t>warranty</t>
+  </si>
+  <si>
+    <t>github</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/PeterBlattner/KCDBtools </t>
   </si>
 </sst>
 </file>
@@ -2091,6 +2097,12 @@
       </c>
     </row>
     <row r="10" spans="3:23" x14ac:dyDescent="0.25">
+      <c r="C10" t="s">
+        <v>444</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>445</v>
+      </c>
       <c r="V10" t="s">
         <v>7</v>
       </c>
@@ -3381,14 +3393,15 @@
     <hyperlink ref="W11" r:id="rId8" xr:uid="{6D9F924D-58BA-4206-8292-DFFCB99795E1}"/>
     <hyperlink ref="W9" r:id="rId9" xr:uid="{A744331A-C32F-4F3A-BA47-EA119444520C}"/>
     <hyperlink ref="D6" r:id="rId10" xr:uid="{2EAE232D-4B86-4EE3-9BB1-549217524CFE}"/>
+    <hyperlink ref="D10" r:id="rId11" xr:uid="{5C957D99-8758-447A-BA6A-A642D019327B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId11"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId12"/>
   <tableParts count="4">
-    <tablePart r:id="rId12"/>
     <tablePart r:id="rId13"/>
     <tablePart r:id="rId14"/>
     <tablePart r:id="rId15"/>
+    <tablePart r:id="rId16"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>